<commit_message>
add basicSAT run and changing format of solution
</commit_message>
<xml_diff>
--- a/2016/results_basicsat.xlsx
+++ b/2016/results_basicsat.xlsx
@@ -10,6 +10,8 @@
     <sheet name="10-S" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="20-S" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="30-S" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="40-S" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="50-S" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2611,7 +2613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2977,6 +2979,3754 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>30_05_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>94</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>300</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>30_05_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>112</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>28.01</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>30_05_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>36</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>25.03</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>30_05_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>56</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>30_05_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>63</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>30_05_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>49</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>58.86</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>30</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30_05_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>81</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>184.39</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30_05_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>86</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30_10_005_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>94</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>30_10_005_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>74</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>30</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>30_10_005_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>112</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>30</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>30_10_005_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>42</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>30_10_005_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>64</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>30_10_005_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>75</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>30</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>30_10_025_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>30_10_025_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>17</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>30</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>30_10_025_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>32</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>30</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>30_10_025_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>30_10_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>107</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>30</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>30_10_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>109</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>30_10_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>30</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>30_10_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>30</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>30_10_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>30</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>30_10_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>30</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>30_10_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>30</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>30-S</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>30_10_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>30</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>solver</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>filename</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Lmax</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>time_s</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gap_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>40_05_005_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>121</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>300</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>40_05_005_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>108</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>40_05_005_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>133</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>40_05_005_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>88</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>300</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>40_05_005_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>114</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>40_05_005_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>152</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>300</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>40_05_025_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>92</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>300</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>40_05_025_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>40_05_025_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>40_05_025_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>74</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>300</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>40_05_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>85</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>138</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>40_05_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>153</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>40_05_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>58</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>18.31</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>40_05_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>77</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>300</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>40_05_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>90</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>300</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>40_05_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>59</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>40_05_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>40</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>92</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>300</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>40_05_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>40</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>118</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>300</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>40_10_005_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>40</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>77</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>40_10_005_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>40</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>55</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>40_10_005_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>115</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>40_10_005_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>164</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>40_10_005_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>40</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>52</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>40_10_005_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>40</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>130</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>40_10_025_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>40</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>40_10_025_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>40</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>81</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>40_10_025_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>136</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>40_10_025_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>40</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>11</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>40_10_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>40</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>94</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>98.17</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>40_10_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>40</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>125</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>40_10_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>40</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>71</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>40_10_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>40</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>4</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>40_10_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>40_10_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>40</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>40_10_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>40</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>11</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>40-S</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>40_10_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>40</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>84</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>261.06</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>solver</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>filename</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Lmax</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>time_s</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gap_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>50_05_005_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>121</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>300</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>50_05_005_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>178</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>300</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>50_05_005_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>182</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>50_05_005_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>50</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>149</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>300</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>50_05_005_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>169</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>300</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>50_05_005_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>176</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>300</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>50_05_025_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>138</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>300</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>50_05_025_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>142</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>50_05_025_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>121</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>300</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>50_05_025_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>50</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>101</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>300</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>50_05_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>50</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>124</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>300</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>50_05_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>50</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>126</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>50_05_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>50</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>82</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>300</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>50_05_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>50</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>122</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>300</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>50_05_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>172</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>300</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>50_05_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>123</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>300</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>50_05_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>108</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>300</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>50_05_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>50</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>157</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>TIMEOUT</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>300</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>50_10_005_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>121</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>50_10_005_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>50</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>78</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>50_10_005_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>50</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>132</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>50_10_005_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>15</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>50_10_005_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>158</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>50_10_005_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>212</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>50_10_025_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>50</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>94</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>50_10_025_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>50</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>22</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>50_10_025_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>50</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>119</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>50_10_025_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>50</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>85</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>50_10_025_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>123</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>150.28</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>50_10_025_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>50</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>77</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>50_10_050_100_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>50</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>33</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>50_10_050_100_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>50</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>132</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>50_10_050_100_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>214</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>50_10_050_125_25_1.GSP</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>50</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>91</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>50_10_050_125_50_1.GSP</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>50</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>82</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>basicsat</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>50-S</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>50_10_050_125_75_1.GSP</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>50</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>125</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>